<commit_message>
Refresh fee and salary datasets
This update regenerates the school data exports after new fee, salary, and student ledger entries were added. It refreshes the generated metadata timestamp, updates the payroll records with September entries and outstanding balances, and adjusts student fee totals, payments, and balances across the current 2026-2027 records.
</commit_message>
<xml_diff>
--- a/source/2026 - 2027 FEE.xlsx
+++ b/source/2026 - 2027 FEE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F11F32D7-9D41-4AE4-AC61-9359E3DBF28A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A39421B-28DF-4BA5-994C-6BB39D92F96B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1ST TERM ACCOUNT" sheetId="14" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="308">
   <si>
     <t>LAST NAME</t>
   </si>
@@ -953,6 +953,15 @@
   <si>
     <t>ABDULAZEEZ FAMILY</t>
   </si>
+  <si>
+    <t>NIP:PAUL ADEDOJA</t>
+  </si>
+  <si>
+    <t>ISLAMIAT YETUNDE TIRIMISIYU</t>
+  </si>
+  <si>
+    <t>ADIGUN AHNAF</t>
+  </si>
 </sst>
 </file>
 
@@ -2136,7 +2145,7 @@
         <v>44</v>
       </c>
       <c r="D7" s="23">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="E7" s="24">
         <v>0</v>
@@ -2159,7 +2168,7 @@
       </c>
       <c r="K7" s="24">
         <f t="shared" si="1"/>
-        <v>18200</v>
+        <v>19500</v>
       </c>
       <c r="L7" s="24">
         <f t="shared" si="2"/>
@@ -2208,14 +2217,14 @@
       </c>
       <c r="Z7" s="24">
         <f t="shared" si="5"/>
-        <v>43130</v>
+        <v>44430</v>
       </c>
       <c r="AA7" s="24">
-        <v>43130</v>
+        <v>20000</v>
       </c>
       <c r="AB7" s="20">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>24430</v>
       </c>
       <c r="AC7" s="24" t="str">
         <f t="shared" si="7"/>
@@ -2231,7 +2240,7 @@
       </c>
       <c r="AF7" s="25" t="str">
         <f t="shared" si="10"/>
-        <v>BONUS</v>
+        <v/>
       </c>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.25">
@@ -2429,11 +2438,11 @@
         <v>44280</v>
       </c>
       <c r="AA9" s="24">
-        <v>16870</v>
+        <v>20000</v>
       </c>
       <c r="AB9" s="20">
         <f t="shared" si="6"/>
-        <v>27410</v>
+        <v>24280</v>
       </c>
       <c r="AC9" s="24" t="str">
         <f t="shared" si="7"/>
@@ -2538,11 +2547,11 @@
         <v>69290</v>
       </c>
       <c r="AA10" s="24">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="AB10" s="20">
         <f t="shared" si="6"/>
-        <v>69290</v>
+        <v>49290</v>
       </c>
       <c r="AC10" s="24" t="str">
         <f t="shared" si="7"/>
@@ -3444,7 +3453,7 @@
         <v>33</v>
       </c>
       <c r="D19" s="23">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="E19" s="24">
         <v>0</v>
@@ -3467,7 +3476,7 @@
       </c>
       <c r="K19" s="24">
         <f t="shared" si="1"/>
-        <v>21000</v>
+        <v>19600</v>
       </c>
       <c r="L19" s="24">
         <f t="shared" si="2"/>
@@ -3475,11 +3484,11 @@
       </c>
       <c r="M19" s="24">
         <f t="shared" si="3"/>
-        <v>1875</v>
+        <v>1750</v>
       </c>
       <c r="N19" s="24">
         <f t="shared" si="4"/>
-        <v>3750</v>
+        <v>3500</v>
       </c>
       <c r="O19" s="24">
         <v>25970</v>
@@ -3516,18 +3525,18 @@
       </c>
       <c r="Z19" s="24">
         <f t="shared" si="5"/>
-        <v>73925</v>
+        <v>72150</v>
       </c>
       <c r="AA19" s="24">
-        <v>51685</v>
+        <v>72150</v>
       </c>
       <c r="AB19" s="20">
         <f t="shared" si="6"/>
-        <v>22240</v>
-      </c>
-      <c r="AC19" s="24" t="str">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="24">
         <f t="shared" si="7"/>
-        <v/>
+        <v>6000</v>
       </c>
       <c r="AD19" s="24" t="str">
         <f t="shared" si="8"/>
@@ -3539,7 +3548,7 @@
       </c>
       <c r="AF19" s="25" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>BONUS</v>
       </c>
     </row>
     <row r="20" spans="1:32" x14ac:dyDescent="0.25">
@@ -3628,11 +3637,11 @@
         <v>76770</v>
       </c>
       <c r="AA20" s="24">
-        <v>0</v>
+        <v>9535</v>
       </c>
       <c r="AB20" s="20">
         <f t="shared" si="6"/>
-        <v>76770</v>
+        <v>67235</v>
       </c>
       <c r="AC20" s="24" t="str">
         <f t="shared" si="7"/>
@@ -4752,7 +4761,7 @@
         <v>49</v>
       </c>
       <c r="D31" s="23">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="E31" s="24">
         <v>0</v>
@@ -4775,7 +4784,7 @@
       </c>
       <c r="K31" s="24">
         <f t="shared" si="1"/>
-        <v>26000</v>
+        <v>24700</v>
       </c>
       <c r="L31" s="24">
         <f t="shared" si="2"/>
@@ -4783,7 +4792,7 @@
       </c>
       <c r="M31" s="24">
         <f t="shared" si="3"/>
-        <v>1000</v>
+        <v>950</v>
       </c>
       <c r="N31" s="24">
         <f t="shared" si="4"/>
@@ -4824,14 +4833,14 @@
       </c>
       <c r="Z31" s="24">
         <f t="shared" si="5"/>
+        <v>41790</v>
+      </c>
+      <c r="AA31" s="24">
         <v>43140</v>
-      </c>
-      <c r="AA31" s="24">
-        <v>0</v>
       </c>
       <c r="AB31" s="20">
         <f t="shared" si="6"/>
-        <v>43140</v>
+        <v>-1350</v>
       </c>
       <c r="AC31" s="24" t="str">
         <f t="shared" si="7"/>
@@ -4847,7 +4856,7 @@
       </c>
       <c r="AF31" s="25" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>BONUS</v>
       </c>
     </row>
     <row r="32" spans="1:32" x14ac:dyDescent="0.25">
@@ -12120,14 +12129,14 @@
         <v>0</v>
       </c>
       <c r="Z98" s="24">
-        <f t="shared" ref="Z98:Z129" si="37">SUM(J98:Y98)</f>
+        <f t="shared" ref="Z98:Z124" si="37">SUM(J98:Y98)</f>
         <v>73925</v>
       </c>
       <c r="AA98" s="24">
         <v>0</v>
       </c>
       <c r="AB98" s="20">
-        <f t="shared" ref="AB98:AB129" si="38">Z98-AA98</f>
+        <f t="shared" ref="AB98:AB124" si="38">Z98-AA98</f>
         <v>73925</v>
       </c>
       <c r="AC98" s="24" t="str">
@@ -14996,8 +15005,8 @@
       <c r="L125" s="28"/>
       <c r="M125" s="28"/>
       <c r="N125" s="28">
-        <f t="shared" ref="N125:AF125" si="42">SUM(N2:N124)</f>
-        <v>259500</v>
+        <f t="shared" ref="N125:AE125" si="42">SUM(N2:N124)</f>
+        <v>259250</v>
       </c>
       <c r="O125" s="28">
         <f t="shared" si="42"/>
@@ -15045,19 +15054,19 @@
       </c>
       <c r="Z125" s="28">
         <f t="shared" si="42"/>
-        <v>7613565</v>
+        <v>7611740</v>
       </c>
       <c r="AA125" s="28">
         <f t="shared" si="42"/>
-        <v>1291035</v>
+        <v>1364175</v>
       </c>
       <c r="AB125" s="28">
         <f t="shared" si="42"/>
-        <v>6322530</v>
+        <v>6247565</v>
       </c>
       <c r="AC125" s="28">
         <f t="shared" si="42"/>
-        <v>12000</v>
+        <v>18000</v>
       </c>
       <c r="AD125" s="28">
         <f t="shared" si="42"/>
@@ -23308,7 +23317,7 @@
       </c>
       <c r="F1" s="36">
         <f>SUM(D2:D1000)</f>
-        <v>1291035</v>
+        <v>1364175</v>
       </c>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
@@ -24130,10 +24139,21 @@
       <c r="X29" s="7"/>
     </row>
     <row r="30" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="7"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="7"/>
+      <c r="A30" s="8">
+        <v>46278</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="D30" s="9">
+        <v>30000</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>254</v>
+      </c>
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
       <c r="H30" s="7"/>
@@ -24155,10 +24175,21 @@
       <c r="X30" s="7"/>
     </row>
     <row r="31" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="7"/>
+      <c r="A31" s="8">
+        <v>46278</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="D31" s="9">
+        <v>43140</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>307</v>
+      </c>
       <c r="F31" s="7"/>
       <c r="G31" s="7"/>
       <c r="H31" s="7"/>
@@ -38184,17 +38215,17 @@
       </c>
       <c r="B2" s="15">
         <f>'1ST TERM ACCOUNT'!AC125</f>
-        <v>12000</v>
+        <v>18000</v>
       </c>
       <c r="C2" s="15">
         <f>B2*0.7</f>
-        <v>8400</v>
+        <v>12600</v>
       </c>
       <c r="D2" s="15"/>
       <c r="E2" s="16"/>
       <c r="F2" s="15">
         <f>$C$2-D2</f>
-        <v>8400</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -38210,7 +38241,7 @@
       <c r="E3" s="16"/>
       <c r="F3" s="15">
         <f>$C$2-(D2+D3)</f>
-        <v>8400</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -38219,14 +38250,14 @@
       </c>
       <c r="B4" s="15">
         <f>B3-B2</f>
-        <v>204000</v>
+        <v>198000</v>
       </c>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="16"/>
       <c r="F4" s="15">
         <f>$C$2-(D2+D3+D4)</f>
-        <v>8400</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -38236,7 +38267,7 @@
       <c r="E5" s="16"/>
       <c r="F5" s="15">
         <f>$C$2-(D2+D3+D4+D5)</f>
-        <v>8400</v>
+        <v>12600</v>
       </c>
       <c r="H5" s="17"/>
     </row>

</xml_diff>

<commit_message>
Update data: students, salary, stock, meta
Refresh generated data and fix multiple records across docs/data and source files. Updated meta.generatedAt and metrics (classCounts, currentOutstanding). Corrected student class typo (PRINARY → PRIMARY) and adjusted several students' paid/balance/latestBalance entries. Modified salary records (name/account/basicSalary/tax/amountPayable/balance), added/removed staff rows and other payroll corrections. Revised stock quantities and recalculated cost/sell totals and profits; removed a placeholder BECE entry. Updated corresponding Excel sources (FEE, SALARY, STOCKS) to match the data changes.
</commit_message>
<xml_diff>
--- a/source/2026 - 2027 FEE.xlsx
+++ b/source/2026 - 2027 FEE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{509D76EA-8349-4561-BD0A-BCB99C049F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F37F3DD-24FE-4729-8069-F8D7965C8870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="837" uniqueCount="406">
   <si>
     <t>LAST NAME</t>
   </si>
@@ -1200,9 +1200,6 @@
     <t>TESTIMONY AYANFE</t>
   </si>
   <si>
-    <t>PRINARY 2</t>
-  </si>
-  <si>
     <t>OLADOSU</t>
   </si>
   <si>
@@ -1252,6 +1249,12 @@
   </si>
   <si>
     <t>MOSES HEPHZIBAH</t>
+  </si>
+  <si>
+    <t>OFURE DIVINE EDIALE</t>
+  </si>
+  <si>
+    <t>OSIGWE FAMILY</t>
   </si>
 </sst>
 </file>
@@ -6089,10 +6092,10 @@
     </row>
     <row r="41" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A41" s="22" t="s">
+        <v>389</v>
+      </c>
+      <c r="B41" s="22" t="s">
         <v>390</v>
-      </c>
-      <c r="B41" s="22" t="s">
-        <v>391</v>
       </c>
       <c r="C41" s="22" t="s">
         <v>44</v>
@@ -9320,7 +9323,7 @@
         <v>368</v>
       </c>
       <c r="C71" s="22" t="s">
-        <v>387</v>
+        <v>48</v>
       </c>
       <c r="D71" s="23">
         <v>0.25</v>
@@ -12544,10 +12547,10 @@
     </row>
     <row r="101" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A101" s="22" t="s">
+        <v>387</v>
+      </c>
+      <c r="B101" s="22" t="s">
         <v>388</v>
-      </c>
-      <c r="B101" s="22" t="s">
-        <v>389</v>
       </c>
       <c r="C101" s="22" t="s">
         <v>44</v>
@@ -14054,10 +14057,10 @@
     </row>
     <row r="115" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A115" s="22" t="s">
+        <v>391</v>
+      </c>
+      <c r="B115" s="22" t="s">
         <v>392</v>
-      </c>
-      <c r="B115" s="22" t="s">
-        <v>393</v>
       </c>
       <c r="C115" s="22" t="s">
         <v>47</v>
@@ -14354,11 +14357,11 @@
         <v>50180</v>
       </c>
       <c r="AA117" s="24">
-        <v>0</v>
+        <v>27120</v>
       </c>
       <c r="AB117" s="20">
         <f>Z117-AA117</f>
-        <v>50180</v>
+        <v>23060</v>
       </c>
       <c r="AC117" s="24" t="str">
         <f>IF(AND($T117=6000, ($T117+$W117-$AB117)&gt;=6000),T117,"")</f>
@@ -14462,11 +14465,11 @@
         <v>72310</v>
       </c>
       <c r="AA118" s="24">
-        <v>0</v>
+        <v>27120</v>
       </c>
       <c r="AB118" s="20">
         <f>Z118-AA118</f>
-        <v>72310</v>
+        <v>45190</v>
       </c>
       <c r="AC118" s="24" t="str">
         <f>IF(AND($T118=6000, ($T118+$W118-$AB118)&gt;=6000),T118,"")</f>
@@ -16620,11 +16623,11 @@
         <v>46880</v>
       </c>
       <c r="AA138" s="24">
-        <v>30000</v>
+        <v>46880</v>
       </c>
       <c r="AB138" s="20">
         <f>Z138-AA138</f>
-        <v>16880</v>
+        <v>0</v>
       </c>
       <c r="AC138" s="24" t="str">
         <f>IF(AND($T138=6000, ($T138+$W138-$AB138)&gt;=6000),T138,"")</f>
@@ -16722,11 +16725,11 @@
       </c>
       <c r="AA139" s="28">
         <f>SUM(AA2:AA138)</f>
-        <v>3390735</v>
+        <v>3461855</v>
       </c>
       <c r="AB139" s="28">
         <f>SUM(AB2:AB138)</f>
-        <v>5479325</v>
+        <v>5408205</v>
       </c>
       <c r="AC139" s="28">
         <f>SUM(AC2:AC138)</f>
@@ -24213,7 +24216,7 @@
     <sortCondition ref="A2:A139"/>
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="AC1:AF10 E139:AF139 AB140:AB996 AB1:AB138">
+  <conditionalFormatting sqref="AC1:AF10 AB1:AB138 E139:AF139 AB140:AB996">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
@@ -24267,7 +24270,7 @@
       </c>
       <c r="F1" s="36">
         <f>SUMIF(E1:E1000, "&lt;&gt;", D1:D1000)</f>
-        <v>3390735</v>
+        <v>3461855</v>
       </c>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
@@ -25067,7 +25070,7 @@
         <v>50000</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="F29" s="7"/>
       <c r="G29" s="7"/>
@@ -25097,13 +25100,13 @@
         <v>250</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="D30" s="9">
         <v>30000</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
@@ -25745,13 +25748,13 @@
         <v>250</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="D48" s="9">
         <v>100000</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="F48" s="7"/>
       <c r="G48" s="7"/>
@@ -26033,13 +26036,13 @@
         <v>250</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D56" s="9">
         <v>22000</v>
       </c>
       <c r="E56" s="7" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="F56" s="7"/>
       <c r="G56" s="7"/>
@@ -26321,13 +26324,13 @@
         <v>250</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D64" s="9">
         <v>124270</v>
       </c>
       <c r="E64" s="7" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F64" s="7"/>
       <c r="G64" s="7"/>
@@ -26399,7 +26402,7 @@
         <v>80000</v>
       </c>
       <c r="E66" s="7" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F66" s="7"/>
       <c r="G66" s="7"/>
@@ -26423,19 +26426,19 @@
     </row>
     <row r="67" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="8">
-        <v>46270</v>
+        <v>46290</v>
       </c>
       <c r="B67" s="7" t="s">
         <v>270</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>272</v>
+        <v>404</v>
       </c>
       <c r="D67" s="9">
-        <v>50000</v>
+        <v>54240</v>
       </c>
       <c r="E67" s="7" t="s">
-        <v>273</v>
+        <v>405</v>
       </c>
       <c r="F67" s="7"/>
       <c r="G67" s="7"/>
@@ -26459,19 +26462,19 @@
     </row>
     <row r="68" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="8">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>315</v>
+        <v>272</v>
       </c>
       <c r="D68" s="9">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="E68" s="7" t="s">
-        <v>329</v>
+        <v>273</v>
       </c>
       <c r="F68" s="7"/>
       <c r="G68" s="7"/>
@@ -26495,19 +26498,19 @@
     </row>
     <row r="69" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="8">
-        <v>46285</v>
+        <v>46280</v>
       </c>
       <c r="B69" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>371</v>
+        <v>315</v>
       </c>
       <c r="D69" s="9">
-        <v>50000</v>
+        <v>100000</v>
       </c>
       <c r="E69" s="7" t="s">
-        <v>383</v>
+        <v>329</v>
       </c>
       <c r="F69" s="7"/>
       <c r="G69" s="7"/>
@@ -26531,19 +26534,19 @@
     </row>
     <row r="70" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="8">
-        <v>46277</v>
+        <v>46285</v>
       </c>
       <c r="B70" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>294</v>
+        <v>371</v>
       </c>
       <c r="D70" s="9">
-        <v>10000</v>
+        <v>50000</v>
       </c>
       <c r="E70" s="7" t="s">
-        <v>297</v>
+        <v>383</v>
       </c>
       <c r="F70" s="7"/>
       <c r="G70" s="7"/>
@@ -26567,19 +26570,19 @@
     </row>
     <row r="71" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="8">
-        <v>46280</v>
+        <v>46277</v>
       </c>
       <c r="B71" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>317</v>
+        <v>294</v>
       </c>
       <c r="D71" s="9">
-        <v>44140</v>
+        <v>10000</v>
       </c>
       <c r="E71" s="7" t="s">
-        <v>348</v>
+        <v>297</v>
       </c>
       <c r="F71" s="7"/>
       <c r="G71" s="7"/>
@@ -26603,19 +26606,19 @@
     </row>
     <row r="72" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8">
-        <v>46266</v>
+        <v>46280</v>
       </c>
       <c r="B72" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>263</v>
+        <v>317</v>
       </c>
       <c r="D72" s="9">
-        <v>50000</v>
+        <v>44140</v>
       </c>
       <c r="E72" s="7" t="s">
-        <v>264</v>
+        <v>348</v>
       </c>
       <c r="F72" s="7"/>
       <c r="G72" s="7"/>
@@ -26639,19 +26642,19 @@
     </row>
     <row r="73" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8">
-        <v>46281</v>
+        <v>46266</v>
       </c>
       <c r="B73" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>345</v>
+        <v>263</v>
       </c>
       <c r="D73" s="9">
-        <v>20000</v>
+        <v>50000</v>
       </c>
       <c r="E73" s="7" t="s">
-        <v>346</v>
+        <v>264</v>
       </c>
       <c r="F73" s="7"/>
       <c r="G73" s="7"/>
@@ -26675,7 +26678,7 @@
     </row>
     <row r="74" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8">
-        <v>46286</v>
+        <v>46281</v>
       </c>
       <c r="B74" s="7" t="s">
         <v>250</v>
@@ -26684,7 +26687,7 @@
         <v>345</v>
       </c>
       <c r="D74" s="9">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="E74" s="7" t="s">
         <v>346</v>
@@ -26711,18 +26714,20 @@
     </row>
     <row r="75" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="8">
-        <v>46279</v>
+        <v>46286</v>
       </c>
       <c r="B75" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>309</v>
+        <v>345</v>
       </c>
       <c r="D75" s="9">
-        <v>36050</v>
-      </c>
-      <c r="E75" s="7"/>
+        <v>10000</v>
+      </c>
+      <c r="E75" s="7" t="s">
+        <v>346</v>
+      </c>
       <c r="F75" s="7"/>
       <c r="G75" s="7"/>
       <c r="H75" s="7"/>
@@ -26745,18 +26750,20 @@
     </row>
     <row r="76" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="8">
-        <v>46279</v>
+        <v>46290</v>
       </c>
       <c r="B76" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>310</v>
+        <v>345</v>
       </c>
       <c r="D76" s="9">
-        <v>100000</v>
-      </c>
-      <c r="E76" s="7"/>
+        <v>16880</v>
+      </c>
+      <c r="E76" s="7" t="s">
+        <v>346</v>
+      </c>
       <c r="F76" s="7"/>
       <c r="G76" s="7"/>
       <c r="H76" s="7"/>
@@ -26782,13 +26789,13 @@
         <v>46279</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D77" s="9">
-        <v>20180</v>
+        <v>36050</v>
       </c>
       <c r="E77" s="7"/>
       <c r="F77" s="7"/>
@@ -26813,18 +26820,18 @@
     </row>
     <row r="78" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="8">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B78" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="C78" s="11" t="s">
-        <v>316</v>
-      </c>
-      <c r="D78" s="12">
-        <v>10000</v>
-      </c>
-      <c r="E78" s="11"/>
+      <c r="C78" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="D78" s="9">
+        <v>100000</v>
+      </c>
+      <c r="E78" s="7"/>
       <c r="F78" s="7"/>
       <c r="G78" s="7"/>
       <c r="H78" s="7"/>
@@ -26847,16 +26854,16 @@
     </row>
     <row r="79" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="8">
-        <v>46281</v>
+        <v>46279</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="D79" s="9">
-        <v>10000</v>
+        <v>20180</v>
       </c>
       <c r="E79" s="7"/>
       <c r="F79" s="7"/>
@@ -26881,18 +26888,18 @@
     </row>
     <row r="80" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="8">
-        <v>46282</v>
+        <v>46280</v>
       </c>
       <c r="B80" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="C80" s="7" t="s">
-        <v>364</v>
-      </c>
-      <c r="D80" s="9">
-        <v>40000</v>
-      </c>
-      <c r="E80" s="7"/>
+      <c r="C80" s="11" t="s">
+        <v>316</v>
+      </c>
+      <c r="D80" s="12">
+        <v>10000</v>
+      </c>
+      <c r="E80" s="11"/>
       <c r="F80" s="7"/>
       <c r="G80" s="7"/>
       <c r="H80" s="7"/>
@@ -26915,16 +26922,16 @@
     </row>
     <row r="81" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="8">
-        <v>46286</v>
+        <v>46281</v>
       </c>
       <c r="B81" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>372</v>
+        <v>316</v>
       </c>
       <c r="D81" s="9">
-        <v>90000</v>
+        <v>10000</v>
       </c>
       <c r="E81" s="7"/>
       <c r="F81" s="7"/>
@@ -26949,13 +26956,13 @@
     </row>
     <row r="82" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="8">
-        <v>46288</v>
+        <v>46282</v>
       </c>
       <c r="B82" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>396</v>
+        <v>364</v>
       </c>
       <c r="D82" s="9">
         <v>40000</v>
@@ -26982,9 +26989,18 @@
       <c r="X82" s="7"/>
     </row>
     <row r="83" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B83" s="7"/>
-      <c r="C83" s="7"/>
-      <c r="D83" s="9"/>
+      <c r="A83" s="8">
+        <v>46286</v>
+      </c>
+      <c r="B83" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="D83" s="9">
+        <v>90000</v>
+      </c>
       <c r="E83" s="7"/>
       <c r="F83" s="7"/>
       <c r="G83" s="7"/>
@@ -27007,9 +27023,18 @@
       <c r="X83" s="7"/>
     </row>
     <row r="84" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B84" s="7"/>
-      <c r="C84" s="7"/>
-      <c r="D84" s="9"/>
+      <c r="A84" s="8">
+        <v>46288</v>
+      </c>
+      <c r="B84" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C84" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="D84" s="9">
+        <v>40000</v>
+      </c>
       <c r="E84" s="7"/>
       <c r="F84" s="7"/>
       <c r="G84" s="7"/>
@@ -39656,8 +39681,8 @@
       <c r="X589" s="7"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F82">
-    <sortCondition ref="E2:E82"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F84">
+    <sortCondition ref="E2:E84"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Update 2026-2027 fee data and balances
Refresh the generated student and metadata files from the 2026-2027 fee workbook. This updates the generated timestamp, reduces the current outstanding total, and corrects several student balances and payment entries based on recent fee adjustments, including a new LESSON FEE PRY extra charge for one record.
</commit_message>
<xml_diff>
--- a/source/2026 - 2027 FEE.xlsx
+++ b/source/2026 - 2027 FEE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A628DB9E-7ACB-4A21-936E-68C36AF4654A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FF3EC81-5496-4243-92AE-9084A62E2CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1ST TERM ACCOUNT" sheetId="14" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="432">
   <si>
     <t>LAST NAME</t>
   </si>
@@ -1221,9 +1221,6 @@
     <t>NIP:MOSES NOAH OLUWASEYI</t>
   </si>
   <si>
-    <t>NIP:ODUNAYO IRETIOLUWA AKINDUN-ALADESAYE AFOLAHANMI VINCENT SCHOOL FE</t>
-  </si>
-  <si>
     <t>NIP:OLADOSU TOSIN ELIZABETH</t>
   </si>
   <si>
@@ -1321,6 +1318,21 @@
   </si>
   <si>
     <t>OLATUNJI FAMILY</t>
+  </si>
+  <si>
+    <t>NIP:ANUOLUWAPO DEBORAH OLADELE-oluwashola Elizabeth and Esther</t>
+  </si>
+  <si>
+    <t>PATIENCE DANIEL</t>
+  </si>
+  <si>
+    <t>OLUWASHOLA FAMILY</t>
+  </si>
+  <si>
+    <t>ISSAH IMOLE</t>
+  </si>
+  <si>
+    <t>NIP:ODUNAYO IRETIOLUWA AKINDUN</t>
   </si>
 </sst>
 </file>
@@ -4192,23 +4204,23 @@
         <v>76770</v>
       </c>
       <c r="AA22" s="24">
-        <v>37535</v>
+        <v>85535</v>
       </c>
       <c r="AB22" s="20">
         <f t="shared" si="6"/>
-        <v>39235</v>
-      </c>
-      <c r="AC22" s="24" t="str">
+        <v>-8765</v>
+      </c>
+      <c r="AC22" s="24">
         <f t="shared" si="7"/>
-        <v/>
+        <v>6000</v>
       </c>
       <c r="AD22" s="24" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="AE22" s="24" t="str">
+      <c r="AE22" s="24">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="AF22" s="25" t="s">
         <v>325</v>
@@ -9679,11 +9691,11 @@
         <v>79830</v>
       </c>
       <c r="AA73" s="24">
-        <v>0</v>
+        <v>40000</v>
       </c>
       <c r="AB73" s="20">
         <f t="shared" si="29"/>
-        <v>79830</v>
+        <v>39830</v>
       </c>
       <c r="AC73" s="24" t="str">
         <f t="shared" si="20"/>
@@ -11643,10 +11655,10 @@
     </row>
     <row r="92" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A92" s="22" t="s">
+        <v>405</v>
+      </c>
+      <c r="B92" s="22" t="s">
         <v>406</v>
-      </c>
-      <c r="B92" s="22" t="s">
-        <v>407</v>
       </c>
       <c r="C92" s="22" t="s">
         <v>332</v>
@@ -14097,11 +14109,11 @@
         <v>45930</v>
       </c>
       <c r="AA114" s="24">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="AB114" s="20">
         <f t="shared" si="39"/>
-        <v>45930</v>
+        <v>25930</v>
       </c>
       <c r="AC114" s="24" t="str">
         <f t="shared" si="30"/>
@@ -14205,11 +14217,11 @@
         <v>57980</v>
       </c>
       <c r="AA115" s="24">
-        <v>0</v>
+        <v>25000</v>
       </c>
       <c r="AB115" s="20">
         <f t="shared" si="39"/>
-        <v>57980</v>
+        <v>32980</v>
       </c>
       <c r="AC115" s="24" t="str">
         <f t="shared" si="30"/>
@@ -15819,14 +15831,14 @@
         <v>1250</v>
       </c>
       <c r="Z130" s="24">
-        <f t="shared" ref="Z130:Z161" si="48">SUM(J130:Y130)</f>
+        <f t="shared" ref="Z130:Z139" si="48">SUM(J130:Y130)</f>
         <v>51530</v>
       </c>
       <c r="AA130" s="24">
         <v>10000</v>
       </c>
       <c r="AB130" s="20">
-        <f t="shared" ref="AB130:AB161" si="49">Z130-AA130</f>
+        <f t="shared" ref="AB130:AB139" si="49">Z130-AA130</f>
         <v>41530</v>
       </c>
       <c r="AC130" s="24" t="str">
@@ -16897,15 +16909,15 @@
       </c>
       <c r="AA140" s="28">
         <f t="shared" si="50"/>
-        <v>4272905</v>
+        <v>4405905</v>
       </c>
       <c r="AB140" s="28">
         <f t="shared" si="50"/>
-        <v>4721065</v>
+        <v>4588065</v>
       </c>
       <c r="AC140" s="28">
         <f t="shared" si="50"/>
-        <v>48000</v>
+        <v>54000</v>
       </c>
       <c r="AD140" s="28">
         <f t="shared" si="50"/>
@@ -24415,7 +24427,7 @@
   <cols>
     <col min="1" max="1" width="14" style="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="107.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="91.140625" style="7" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.5703125" style="9" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.28515625" style="7" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.7109375" style="7" bestFit="1" customWidth="1"/>
@@ -24442,7 +24454,7 @@
       </c>
       <c r="F1" s="36">
         <f>SUMIF(E1:E1000, "&lt;&gt;", D1:D1000)</f>
-        <v>4272905</v>
+        <v>4405905</v>
       </c>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
@@ -24870,19 +24882,19 @@
     </row>
     <row r="19" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
-        <v>46278</v>
+        <v>46295</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="D19" s="9">
-        <v>62230</v>
+        <v>48000</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>303</v>
+        <v>254</v>
       </c>
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
@@ -24906,19 +24918,19 @@
     </row>
     <row r="20" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8">
-        <v>46271</v>
+        <v>46278</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>267</v>
+        <v>301</v>
       </c>
       <c r="D20" s="9">
-        <v>60000</v>
+        <v>62230</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>268</v>
+        <v>303</v>
       </c>
       <c r="F20" s="7"/>
       <c r="G20" s="7"/>
@@ -24942,19 +24954,19 @@
     </row>
     <row r="21" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8">
-        <v>46286</v>
+        <v>46271</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>376</v>
+        <v>267</v>
       </c>
       <c r="D21" s="9">
-        <v>27000</v>
+        <v>60000</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>379</v>
+        <v>268</v>
       </c>
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
@@ -24981,13 +24993,13 @@
         <v>46286</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D22" s="9">
-        <v>16140</v>
+        <v>27000</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>379</v>
@@ -25014,19 +25026,19 @@
     </row>
     <row r="23" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
-        <v>46280</v>
+        <v>46286</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>321</v>
+        <v>377</v>
       </c>
       <c r="D23" s="9">
-        <v>40000</v>
+        <v>16140</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>327</v>
+        <v>379</v>
       </c>
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
@@ -25050,19 +25062,19 @@
     </row>
     <row r="24" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8">
-        <v>46278</v>
+        <v>46280</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>306</v>
+        <v>321</v>
       </c>
       <c r="D24" s="9">
-        <v>43140</v>
+        <v>40000</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>307</v>
+        <v>327</v>
       </c>
       <c r="F24" s="7"/>
       <c r="G24" s="7"/>
@@ -25086,19 +25098,19 @@
     </row>
     <row r="25" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
-        <v>46280</v>
+        <v>46278</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>319</v>
+        <v>306</v>
       </c>
       <c r="D25" s="9">
-        <v>60000</v>
+        <v>43140</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>333</v>
+        <v>307</v>
       </c>
       <c r="F25" s="7"/>
       <c r="G25" s="7"/>
@@ -25122,19 +25134,19 @@
     </row>
     <row r="26" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8">
-        <v>46265</v>
+        <v>46280</v>
       </c>
       <c r="B26" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>260</v>
+        <v>319</v>
       </c>
       <c r="D26" s="9">
-        <v>50430</v>
+        <v>60000</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>262</v>
+        <v>333</v>
       </c>
       <c r="F26" s="7"/>
       <c r="G26" s="7"/>
@@ -25158,19 +25170,19 @@
     </row>
     <row r="27" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8">
-        <v>46276</v>
+        <v>46265</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>291</v>
+        <v>260</v>
       </c>
       <c r="D27" s="9">
-        <v>28000</v>
+        <v>50430</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>298</v>
+        <v>262</v>
       </c>
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
@@ -25194,7 +25206,7 @@
     </row>
     <row r="28" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8">
-        <v>46280</v>
+        <v>46276</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>250</v>
@@ -25203,7 +25215,7 @@
         <v>291</v>
       </c>
       <c r="D28" s="9">
-        <v>15140</v>
+        <v>28000</v>
       </c>
       <c r="E28" s="7" t="s">
         <v>298</v>
@@ -25230,19 +25242,19 @@
     </row>
     <row r="29" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>365</v>
+        <v>291</v>
       </c>
       <c r="D29" s="9">
-        <v>50000</v>
+        <v>15140</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>402</v>
+        <v>298</v>
       </c>
       <c r="F29" s="7"/>
       <c r="G29" s="7"/>
@@ -25266,19 +25278,19 @@
     </row>
     <row r="30" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8">
-        <v>46287</v>
+        <v>46283</v>
       </c>
       <c r="B30" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>394</v>
+        <v>365</v>
       </c>
       <c r="D30" s="9">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
@@ -25302,19 +25314,19 @@
     </row>
     <row r="31" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8">
-        <v>46278</v>
+        <v>46287</v>
       </c>
       <c r="B31" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>299</v>
+        <v>431</v>
       </c>
       <c r="D31" s="9">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>302</v>
+        <v>399</v>
       </c>
       <c r="F31" s="7"/>
       <c r="G31" s="7"/>
@@ -25338,19 +25350,19 @@
     </row>
     <row r="32" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="8">
-        <v>46270</v>
+        <v>46278</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>269</v>
+        <v>299</v>
       </c>
       <c r="D32" s="9">
-        <v>79020</v>
+        <v>50000</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>275</v>
+        <v>302</v>
       </c>
       <c r="F32" s="7"/>
       <c r="G32" s="7"/>
@@ -25374,19 +25386,19 @@
     </row>
     <row r="33" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8">
-        <v>46238</v>
+        <v>46270</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>249</v>
+        <v>269</v>
       </c>
       <c r="D33" s="9">
-        <v>48000</v>
+        <v>79020</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>251</v>
+        <v>275</v>
       </c>
       <c r="F33" s="7"/>
       <c r="G33" s="7"/>
@@ -25410,7 +25422,7 @@
     </row>
     <row r="34" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8">
-        <v>46282</v>
+        <v>46238</v>
       </c>
       <c r="B34" s="7" t="s">
         <v>250</v>
@@ -25419,7 +25431,7 @@
         <v>249</v>
       </c>
       <c r="D34" s="9">
-        <v>35180</v>
+        <v>48000</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>251</v>
@@ -25446,19 +25458,19 @@
     </row>
     <row r="35" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8">
-        <v>46270</v>
+        <v>46282</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>271</v>
+        <v>249</v>
       </c>
       <c r="D35" s="9">
-        <v>42350</v>
+        <v>35180</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>274</v>
+        <v>251</v>
       </c>
       <c r="F35" s="7"/>
       <c r="G35" s="7"/>
@@ -25482,7 +25494,7 @@
     </row>
     <row r="36" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8">
-        <v>46282</v>
+        <v>46270</v>
       </c>
       <c r="B36" s="7" t="s">
         <v>270</v>
@@ -25491,7 +25503,7 @@
         <v>271</v>
       </c>
       <c r="D36" s="9">
-        <v>40000</v>
+        <v>42350</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>274</v>
@@ -25518,19 +25530,19 @@
     </row>
     <row r="37" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="8">
-        <v>46279</v>
+        <v>46282</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>310</v>
+        <v>271</v>
       </c>
       <c r="D37" s="9">
-        <v>100000</v>
+        <v>40000</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>419</v>
+        <v>274</v>
       </c>
       <c r="F37" s="7"/>
       <c r="G37" s="7"/>
@@ -25554,19 +25566,19 @@
     </row>
     <row r="38" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="8">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B38" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="C38" s="11" t="s">
-        <v>323</v>
-      </c>
-      <c r="D38" s="12">
-        <v>40000</v>
-      </c>
-      <c r="E38" s="11" t="s">
-        <v>328</v>
+      <c r="C38" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="D38" s="9">
+        <v>100000</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>418</v>
       </c>
       <c r="F38" s="7"/>
       <c r="G38" s="7"/>
@@ -25590,18 +25602,18 @@
     </row>
     <row r="39" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8">
-        <v>46289</v>
+        <v>46280</v>
       </c>
       <c r="B39" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="C39" s="11" t="s">
         <v>323</v>
       </c>
-      <c r="D39" s="9">
-        <v>88000</v>
-      </c>
-      <c r="E39" s="7" t="s">
+      <c r="D39" s="12">
+        <v>40000</v>
+      </c>
+      <c r="E39" s="11" t="s">
         <v>328</v>
       </c>
       <c r="F39" s="7"/>
@@ -25626,19 +25638,19 @@
     </row>
     <row r="40" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8">
-        <v>46273</v>
+        <v>46289</v>
       </c>
       <c r="B40" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>277</v>
+        <v>323</v>
       </c>
       <c r="D40" s="9">
-        <v>33000</v>
+        <v>88000</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>282</v>
+        <v>328</v>
       </c>
       <c r="F40" s="7"/>
       <c r="G40" s="7"/>
@@ -25665,13 +25677,13 @@
         <v>46273</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D41" s="9">
-        <v>6840</v>
+        <v>33000</v>
       </c>
       <c r="E41" s="7" t="s">
         <v>282</v>
@@ -25698,7 +25710,7 @@
     </row>
     <row r="42" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8">
-        <v>46281</v>
+        <v>46273</v>
       </c>
       <c r="B42" s="7" t="s">
         <v>270</v>
@@ -25707,12 +25719,12 @@
         <v>278</v>
       </c>
       <c r="D42" s="9">
-        <v>5300</v>
+        <v>6840</v>
       </c>
       <c r="E42" s="7" t="s">
         <v>282</v>
       </c>
-      <c r="F42" s="11"/>
+      <c r="F42" s="7"/>
       <c r="G42" s="7"/>
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
@@ -25748,7 +25760,7 @@
       <c r="E43" s="7" t="s">
         <v>282</v>
       </c>
-      <c r="F43" s="7"/>
+      <c r="F43" s="11"/>
       <c r="G43" s="7"/>
       <c r="H43" s="7"/>
       <c r="I43" s="7"/>
@@ -25770,19 +25782,19 @@
     </row>
     <row r="44" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8">
-        <v>46273</v>
+        <v>46281</v>
       </c>
       <c r="B44" s="7" t="s">
         <v>270</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D44" s="9">
-        <v>200000</v>
+        <v>5300</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F44" s="7"/>
       <c r="G44" s="7"/>
@@ -25806,19 +25818,19 @@
     </row>
     <row r="45" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="8">
-        <v>46286</v>
+        <v>46273</v>
       </c>
       <c r="B45" s="7" t="s">
         <v>270</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>378</v>
+        <v>279</v>
       </c>
       <c r="D45" s="9">
-        <v>56930</v>
+        <v>200000</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>384</v>
+        <v>281</v>
       </c>
       <c r="F45" s="7"/>
       <c r="G45" s="7"/>
@@ -25842,19 +25854,19 @@
     </row>
     <row r="46" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="8">
-        <v>46264</v>
+        <v>46286</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>256</v>
+        <v>378</v>
       </c>
       <c r="D46" s="9">
-        <v>51930</v>
+        <v>56930</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>257</v>
+        <v>384</v>
       </c>
       <c r="F46" s="7"/>
       <c r="G46" s="7"/>
@@ -25878,19 +25890,19 @@
     </row>
     <row r="47" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="8">
-        <v>46279</v>
+        <v>46264</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>312</v>
+        <v>256</v>
       </c>
       <c r="D47" s="9">
-        <v>25000</v>
+        <v>51930</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>313</v>
+        <v>257</v>
       </c>
       <c r="F47" s="7"/>
       <c r="G47" s="7"/>
@@ -25914,19 +25926,19 @@
     </row>
     <row r="48" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>342</v>
+        <v>312</v>
       </c>
       <c r="D48" s="9">
-        <v>50000</v>
+        <v>25000</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>343</v>
+        <v>313</v>
       </c>
       <c r="F48" s="7"/>
       <c r="G48" s="7"/>
@@ -25950,19 +25962,19 @@
     </row>
     <row r="49" spans="1:24" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="8">
-        <v>46288</v>
+        <v>46280</v>
       </c>
       <c r="B49" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>396</v>
+        <v>342</v>
       </c>
       <c r="D49" s="9">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>399</v>
+        <v>343</v>
       </c>
       <c r="F49" s="7"/>
       <c r="G49" s="11"/>
@@ -25986,19 +25998,19 @@
     </row>
     <row r="50" spans="1:24" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="8">
-        <v>46280</v>
+        <v>46288</v>
       </c>
       <c r="B50" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>314</v>
+        <v>395</v>
       </c>
       <c r="D50" s="9">
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="E50" s="7" t="s">
-        <v>369</v>
+        <v>398</v>
       </c>
       <c r="F50" s="7"/>
       <c r="G50" s="11"/>
@@ -26027,14 +26039,14 @@
       <c r="B51" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="C51" s="11" t="s">
-        <v>316</v>
-      </c>
-      <c r="D51" s="12">
-        <v>10000</v>
-      </c>
-      <c r="E51" s="11" t="s">
-        <v>420</v>
+      <c r="C51" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="D51" s="9">
+        <v>30000</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>369</v>
       </c>
       <c r="F51" s="7"/>
       <c r="G51" s="11"/>
@@ -26058,19 +26070,19 @@
     </row>
     <row r="52" spans="1:24" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="8">
-        <v>46281</v>
+        <v>46294</v>
       </c>
       <c r="B52" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>316</v>
+        <v>422</v>
       </c>
       <c r="D52" s="9">
-        <v>10000</v>
+        <v>40000</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>420</v>
+        <v>369</v>
       </c>
       <c r="F52" s="7"/>
       <c r="G52" s="11"/>
@@ -26093,20 +26105,20 @@
       <c r="X52" s="11"/>
     </row>
     <row r="53" spans="1:24" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="10">
-        <v>46271</v>
-      </c>
-      <c r="B53" s="11" t="s">
+      <c r="A53" s="8">
+        <v>46280</v>
+      </c>
+      <c r="B53" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>276</v>
+        <v>316</v>
       </c>
       <c r="D53" s="12">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>283</v>
+        <v>419</v>
       </c>
       <c r="F53" s="7"/>
       <c r="G53" s="11"/>
@@ -26130,19 +26142,19 @@
     </row>
     <row r="54" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="8">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="B54" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>276</v>
+        <v>316</v>
       </c>
       <c r="D54" s="9">
-        <v>9640</v>
+        <v>10000</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>283</v>
+        <v>419</v>
       </c>
       <c r="F54" s="7"/>
       <c r="G54" s="7"/>
@@ -26166,19 +26178,19 @@
     </row>
     <row r="55" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="8">
-        <v>46292</v>
+        <v>46296</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>410</v>
+        <v>428</v>
       </c>
       <c r="D55" s="9">
-        <v>50000</v>
+        <v>40000</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>414</v>
+        <v>430</v>
       </c>
       <c r="F55" s="7"/>
       <c r="G55" s="7"/>
@@ -26201,22 +26213,22 @@
       <c r="X55" s="7"/>
     </row>
     <row r="56" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="8">
-        <v>46280</v>
-      </c>
-      <c r="B56" s="7" t="s">
+      <c r="A56" s="10">
+        <v>46271</v>
+      </c>
+      <c r="B56" s="11" t="s">
         <v>250</v>
       </c>
-      <c r="C56" s="7" t="s">
-        <v>339</v>
-      </c>
-      <c r="D56" s="9">
-        <v>65160</v>
-      </c>
-      <c r="E56" s="7" t="s">
-        <v>340</v>
-      </c>
-      <c r="F56" s="11"/>
+      <c r="C56" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="D56" s="12">
+        <v>20000</v>
+      </c>
+      <c r="E56" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="F56" s="7"/>
       <c r="G56" s="7"/>
       <c r="H56" s="7"/>
       <c r="I56" s="7"/>
@@ -26238,21 +26250,21 @@
     </row>
     <row r="57" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="8">
-        <v>46280</v>
+        <v>46278</v>
       </c>
       <c r="B57" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>339</v>
+        <v>276</v>
       </c>
       <c r="D57" s="9">
-        <v>35890</v>
+        <v>9640</v>
       </c>
       <c r="E57" s="7" t="s">
-        <v>341</v>
-      </c>
-      <c r="F57" s="11"/>
+        <v>283</v>
+      </c>
+      <c r="F57" s="7"/>
       <c r="G57" s="7"/>
       <c r="H57" s="7"/>
       <c r="I57" s="7"/>
@@ -26274,19 +26286,19 @@
     </row>
     <row r="58" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="8">
-        <v>46280</v>
+        <v>46292</v>
       </c>
       <c r="B58" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>344</v>
+        <v>409</v>
       </c>
       <c r="D58" s="9">
         <v>50000</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>347</v>
+        <v>413</v>
       </c>
       <c r="F58" s="7"/>
       <c r="G58" s="7"/>
@@ -26310,21 +26322,21 @@
     </row>
     <row r="59" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="8">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="B59" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>308</v>
+        <v>339</v>
       </c>
       <c r="D59" s="9">
-        <v>116000</v>
+        <v>65160</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>363</v>
-      </c>
-      <c r="F59" s="7"/>
+        <v>340</v>
+      </c>
+      <c r="F59" s="11"/>
       <c r="G59" s="7"/>
       <c r="H59" s="7"/>
       <c r="I59" s="7"/>
@@ -26346,21 +26358,21 @@
     </row>
     <row r="60" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="8">
-        <v>46287</v>
+        <v>46280</v>
       </c>
       <c r="B60" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>393</v>
+        <v>339</v>
       </c>
       <c r="D60" s="9">
-        <v>22000</v>
+        <v>35890</v>
       </c>
       <c r="E60" s="7" t="s">
-        <v>403</v>
-      </c>
-      <c r="F60" s="7"/>
+        <v>341</v>
+      </c>
+      <c r="F60" s="11"/>
       <c r="G60" s="7"/>
       <c r="H60" s="7"/>
       <c r="I60" s="7"/>
@@ -26382,19 +26394,19 @@
     </row>
     <row r="61" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="8">
-        <v>46284</v>
+        <v>46280</v>
       </c>
       <c r="B61" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>370</v>
+        <v>344</v>
       </c>
       <c r="D61" s="9">
         <v>50000</v>
       </c>
       <c r="E61" s="7" t="s">
-        <v>382</v>
+        <v>347</v>
       </c>
       <c r="F61" s="7"/>
       <c r="G61" s="7"/>
@@ -26418,19 +26430,19 @@
     </row>
     <row r="62" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="8">
-        <v>46285</v>
+        <v>46279</v>
       </c>
       <c r="B62" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>370</v>
+        <v>308</v>
       </c>
       <c r="D62" s="9">
-        <v>50000</v>
+        <v>116000</v>
       </c>
       <c r="E62" s="7" t="s">
-        <v>382</v>
+        <v>363</v>
       </c>
       <c r="F62" s="7"/>
       <c r="G62" s="7"/>
@@ -26454,19 +26466,19 @@
     </row>
     <row r="63" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="8">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="B63" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>372</v>
+        <v>393</v>
       </c>
       <c r="D63" s="9">
-        <v>90000</v>
+        <v>22000</v>
       </c>
       <c r="E63" s="7" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
       <c r="F63" s="7"/>
       <c r="G63" s="7"/>
@@ -26490,19 +26502,19 @@
     </row>
     <row r="64" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="8">
-        <v>46286</v>
+        <v>46294</v>
       </c>
       <c r="B64" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>375</v>
+        <v>421</v>
       </c>
       <c r="D64" s="9">
-        <v>50000</v>
+        <v>65000</v>
       </c>
       <c r="E64" s="7" t="s">
-        <v>381</v>
+        <v>402</v>
       </c>
       <c r="F64" s="7"/>
       <c r="G64" s="7"/>
@@ -26526,19 +26538,19 @@
     </row>
     <row r="65" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="8">
-        <v>46277</v>
+        <v>46284</v>
       </c>
       <c r="B65" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>292</v>
+        <v>370</v>
       </c>
       <c r="D65" s="9">
-        <v>95000</v>
+        <v>50000</v>
       </c>
       <c r="E65" s="7" t="s">
-        <v>293</v>
+        <v>382</v>
       </c>
       <c r="F65" s="7"/>
       <c r="G65" s="7"/>
@@ -26562,19 +26574,19 @@
     </row>
     <row r="66" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="8">
-        <v>46293</v>
+        <v>46285</v>
       </c>
       <c r="B66" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>412</v>
+        <v>370</v>
       </c>
       <c r="D66" s="9">
-        <v>80000</v>
+        <v>50000</v>
       </c>
       <c r="E66" s="7" t="s">
-        <v>416</v>
+        <v>382</v>
       </c>
       <c r="F66" s="7"/>
       <c r="G66" s="7"/>
@@ -26598,19 +26610,19 @@
     </row>
     <row r="67" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="8">
-        <v>46280</v>
+        <v>46286</v>
       </c>
       <c r="B67" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>322</v>
+        <v>372</v>
       </c>
       <c r="D67" s="9">
-        <v>27900</v>
+        <v>90000</v>
       </c>
       <c r="E67" s="7" t="s">
-        <v>324</v>
+        <v>407</v>
       </c>
       <c r="F67" s="7"/>
       <c r="G67" s="7"/>
@@ -26634,19 +26646,19 @@
     </row>
     <row r="68" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="8">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="B68" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>395</v>
+        <v>375</v>
       </c>
       <c r="D68" s="9">
-        <v>40000</v>
+        <v>50000</v>
       </c>
       <c r="E68" s="7" t="s">
-        <v>421</v>
+        <v>381</v>
       </c>
       <c r="F68" s="7"/>
       <c r="G68" s="7"/>
@@ -26670,19 +26682,19 @@
     </row>
     <row r="69" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="8">
-        <v>46275</v>
+        <v>46277</v>
       </c>
       <c r="B69" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="D69" s="9">
-        <v>24700</v>
+        <v>95000</v>
       </c>
       <c r="E69" s="7" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="F69" s="7"/>
       <c r="G69" s="7"/>
@@ -26706,19 +26718,19 @@
     </row>
     <row r="70" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="8">
-        <v>46279</v>
+        <v>46293</v>
       </c>
       <c r="B70" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>286</v>
+        <v>411</v>
       </c>
       <c r="D70" s="9">
-        <v>20000</v>
+        <v>80000</v>
       </c>
       <c r="E70" s="7" t="s">
-        <v>287</v>
+        <v>415</v>
       </c>
       <c r="F70" s="7"/>
       <c r="G70" s="7"/>
@@ -26742,19 +26754,19 @@
     </row>
     <row r="71" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="8">
-        <v>46293</v>
+        <v>46280</v>
       </c>
       <c r="B71" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>295</v>
+        <v>322</v>
       </c>
       <c r="D71" s="9">
-        <v>30000</v>
+        <v>27900</v>
       </c>
       <c r="E71" s="7" t="s">
-        <v>415</v>
+        <v>324</v>
       </c>
       <c r="F71" s="7"/>
       <c r="G71" s="7"/>
@@ -26784,13 +26796,13 @@
         <v>250</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="D72" s="9">
-        <v>124270</v>
+        <v>40000</v>
       </c>
       <c r="E72" s="7" t="s">
-        <v>398</v>
+        <v>420</v>
       </c>
       <c r="F72" s="7"/>
       <c r="G72" s="7"/>
@@ -26813,20 +26825,20 @@
       <c r="X72" s="7"/>
     </row>
     <row r="73" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="10">
+      <c r="A73" s="8">
         <v>46275</v>
       </c>
-      <c r="B73" s="11" t="s">
+      <c r="B73" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="C73" s="11" t="s">
-        <v>285</v>
-      </c>
-      <c r="D73" s="12">
-        <v>33140</v>
-      </c>
-      <c r="E73" s="11" t="s">
-        <v>284</v>
+      <c r="C73" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="D73" s="9">
+        <v>24700</v>
+      </c>
+      <c r="E73" s="7" t="s">
+        <v>287</v>
       </c>
       <c r="F73" s="7"/>
       <c r="G73" s="7"/>
@@ -26850,19 +26862,19 @@
     </row>
     <row r="74" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8">
-        <v>46286</v>
+        <v>46279</v>
       </c>
       <c r="B74" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>374</v>
+        <v>286</v>
       </c>
       <c r="D74" s="9">
-        <v>80000</v>
+        <v>20000</v>
       </c>
       <c r="E74" s="7" t="s">
-        <v>401</v>
+        <v>287</v>
       </c>
       <c r="F74" s="7"/>
       <c r="G74" s="7"/>
@@ -26886,19 +26898,19 @@
     </row>
     <row r="75" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="8">
-        <v>46292</v>
+        <v>46294</v>
       </c>
       <c r="B75" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>409</v>
+        <v>424</v>
       </c>
       <c r="D75" s="9">
-        <v>30000</v>
+        <v>140000</v>
       </c>
       <c r="E75" s="7" t="s">
-        <v>413</v>
+        <v>426</v>
       </c>
       <c r="F75" s="7"/>
       <c r="G75" s="7"/>
@@ -26922,19 +26934,19 @@
     </row>
     <row r="76" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="8">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>404</v>
+        <v>295</v>
       </c>
       <c r="D76" s="9">
-        <v>54240</v>
+        <v>30000</v>
       </c>
       <c r="E76" s="7" t="s">
-        <v>405</v>
+        <v>414</v>
       </c>
       <c r="F76" s="7"/>
       <c r="G76" s="7"/>
@@ -26958,19 +26970,19 @@
     </row>
     <row r="77" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="8">
-        <v>46279</v>
+        <v>46288</v>
       </c>
       <c r="B77" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>309</v>
+        <v>396</v>
       </c>
       <c r="D77" s="9">
-        <v>36050</v>
+        <v>124270</v>
       </c>
       <c r="E77" s="7" t="s">
-        <v>418</v>
+        <v>397</v>
       </c>
       <c r="F77" s="7"/>
       <c r="G77" s="7"/>
@@ -26993,20 +27005,20 @@
       <c r="X77" s="7"/>
     </row>
     <row r="78" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="8">
-        <v>46270</v>
-      </c>
-      <c r="B78" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="C78" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="D78" s="9">
-        <v>50000</v>
-      </c>
-      <c r="E78" s="7" t="s">
-        <v>273</v>
+      <c r="A78" s="10">
+        <v>46275</v>
+      </c>
+      <c r="B78" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="C78" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="D78" s="12">
+        <v>33140</v>
+      </c>
+      <c r="E78" s="11" t="s">
+        <v>284</v>
       </c>
       <c r="F78" s="7"/>
       <c r="G78" s="7"/>
@@ -27030,19 +27042,19 @@
     </row>
     <row r="79" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="8">
-        <v>46280</v>
+        <v>46295</v>
       </c>
       <c r="B79" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>315</v>
+        <v>427</v>
       </c>
       <c r="D79" s="9">
-        <v>100000</v>
+        <v>45000</v>
       </c>
       <c r="E79" s="7" t="s">
-        <v>329</v>
+        <v>429</v>
       </c>
       <c r="F79" s="7"/>
       <c r="G79" s="7"/>
@@ -27066,19 +27078,19 @@
     </row>
     <row r="80" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="8">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="B80" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="D80" s="9">
-        <v>50000</v>
+        <v>80000</v>
       </c>
       <c r="E80" s="7" t="s">
-        <v>383</v>
+        <v>400</v>
       </c>
       <c r="F80" s="7"/>
       <c r="G80" s="7"/>
@@ -27102,19 +27114,19 @@
     </row>
     <row r="81" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="8">
-        <v>46277</v>
+        <v>46292</v>
       </c>
       <c r="B81" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>294</v>
+        <v>408</v>
       </c>
       <c r="D81" s="9">
-        <v>10000</v>
+        <v>30000</v>
       </c>
       <c r="E81" s="7" t="s">
-        <v>297</v>
+        <v>412</v>
       </c>
       <c r="F81" s="7"/>
       <c r="G81" s="7"/>
@@ -27138,19 +27150,19 @@
     </row>
     <row r="82" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="8">
-        <v>46280</v>
+        <v>46290</v>
       </c>
       <c r="B82" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>317</v>
+        <v>403</v>
       </c>
       <c r="D82" s="9">
-        <v>44140</v>
+        <v>54240</v>
       </c>
       <c r="E82" s="7" t="s">
-        <v>348</v>
+        <v>404</v>
       </c>
       <c r="F82" s="7"/>
       <c r="G82" s="7"/>
@@ -27174,16 +27186,16 @@
     </row>
     <row r="83" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="8">
-        <v>46293</v>
+        <v>46279</v>
       </c>
       <c r="B83" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>411</v>
+        <v>309</v>
       </c>
       <c r="D83" s="9">
-        <v>50000</v>
+        <v>36050</v>
       </c>
       <c r="E83" s="7" t="s">
         <v>417</v>
@@ -27210,19 +27222,19 @@
     </row>
     <row r="84" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="8">
-        <v>46266</v>
+        <v>46270</v>
       </c>
       <c r="B84" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="D84" s="9">
         <v>50000</v>
       </c>
       <c r="E84" s="7" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="F84" s="7"/>
       <c r="G84" s="7"/>
@@ -27246,19 +27258,19 @@
     </row>
     <row r="85" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="8">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="B85" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>345</v>
+        <v>315</v>
       </c>
       <c r="D85" s="9">
-        <v>20000</v>
+        <v>100000</v>
       </c>
       <c r="E85" s="7" t="s">
-        <v>346</v>
+        <v>329</v>
       </c>
       <c r="F85" s="7"/>
       <c r="G85" s="7"/>
@@ -27282,19 +27294,19 @@
     </row>
     <row r="86" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="8">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="B86" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>345</v>
+        <v>371</v>
       </c>
       <c r="D86" s="9">
-        <v>10000</v>
+        <v>50000</v>
       </c>
       <c r="E86" s="7" t="s">
-        <v>346</v>
+        <v>383</v>
       </c>
       <c r="F86" s="7"/>
       <c r="G86" s="7"/>
@@ -27318,19 +27330,19 @@
     </row>
     <row r="87" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="8">
-        <v>46290</v>
+        <v>46277</v>
       </c>
       <c r="B87" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>345</v>
+        <v>294</v>
       </c>
       <c r="D87" s="9">
-        <v>16880</v>
+        <v>10000</v>
       </c>
       <c r="E87" s="7" t="s">
-        <v>346</v>
+        <v>297</v>
       </c>
       <c r="F87" s="7"/>
       <c r="G87" s="7"/>
@@ -27354,18 +27366,20 @@
     </row>
     <row r="88" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="8">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="B88" s="7" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="D88" s="9">
-        <v>20180</v>
-      </c>
-      <c r="E88" s="7"/>
+        <v>44140</v>
+      </c>
+      <c r="E88" s="7" t="s">
+        <v>348</v>
+      </c>
       <c r="F88" s="7"/>
       <c r="G88" s="7"/>
       <c r="H88" s="7"/>
@@ -27388,18 +27402,20 @@
     </row>
     <row r="89" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="8">
-        <v>46282</v>
+        <v>46294</v>
       </c>
       <c r="B89" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>364</v>
+        <v>423</v>
       </c>
       <c r="D89" s="9">
         <v>40000</v>
       </c>
-      <c r="E89" s="7"/>
+      <c r="E89" s="7" t="s">
+        <v>425</v>
+      </c>
       <c r="F89" s="7"/>
       <c r="G89" s="7"/>
       <c r="H89" s="7"/>
@@ -27422,19 +27438,19 @@
     </row>
     <row r="90" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="8">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="B90" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C90" s="7" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="D90" s="9">
-        <v>65000</v>
+        <v>50000</v>
       </c>
       <c r="E90" s="7" t="s">
-        <v>403</v>
+        <v>416</v>
       </c>
       <c r="F90" s="7"/>
       <c r="G90" s="7"/>
@@ -27458,19 +27474,19 @@
     </row>
     <row r="91" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="8">
-        <v>46294</v>
+        <v>46266</v>
       </c>
       <c r="B91" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>423</v>
+        <v>263</v>
       </c>
       <c r="D91" s="9">
-        <v>40000</v>
+        <v>50000</v>
       </c>
       <c r="E91" s="7" t="s">
-        <v>369</v>
+        <v>264</v>
       </c>
       <c r="F91" s="7"/>
       <c r="G91" s="7"/>
@@ -27494,19 +27510,19 @@
     </row>
     <row r="92" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="8">
-        <v>46294</v>
+        <v>46281</v>
       </c>
       <c r="B92" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>424</v>
+        <v>345</v>
       </c>
       <c r="D92" s="9">
-        <v>40000</v>
+        <v>20000</v>
       </c>
       <c r="E92" s="7" t="s">
-        <v>426</v>
+        <v>346</v>
       </c>
       <c r="F92" s="7"/>
       <c r="G92" s="7"/>
@@ -27530,19 +27546,19 @@
     </row>
     <row r="93" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="8">
-        <v>46294</v>
+        <v>46286</v>
       </c>
       <c r="B93" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>425</v>
+        <v>345</v>
       </c>
       <c r="D93" s="9">
-        <v>140000</v>
+        <v>10000</v>
       </c>
       <c r="E93" s="7" t="s">
-        <v>427</v>
+        <v>346</v>
       </c>
       <c r="F93" s="7"/>
       <c r="G93" s="7"/>
@@ -27565,10 +27581,21 @@
       <c r="X93" s="7"/>
     </row>
     <row r="94" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B94" s="7"/>
-      <c r="C94" s="7"/>
-      <c r="D94" s="9"/>
-      <c r="E94" s="7"/>
+      <c r="A94" s="8">
+        <v>46290</v>
+      </c>
+      <c r="B94" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C94" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="D94" s="9">
+        <v>16880</v>
+      </c>
+      <c r="E94" s="7" t="s">
+        <v>346</v>
+      </c>
       <c r="F94" s="7"/>
       <c r="G94" s="7"/>
       <c r="H94" s="7"/>
@@ -27590,9 +27617,18 @@
       <c r="X94" s="7"/>
     </row>
     <row r="95" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B95" s="7"/>
-      <c r="C95" s="7"/>
-      <c r="D95" s="9"/>
+      <c r="A95" s="8">
+        <v>46279</v>
+      </c>
+      <c r="B95" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="C95" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="D95" s="9">
+        <v>20180</v>
+      </c>
       <c r="E95" s="7"/>
       <c r="F95" s="7"/>
       <c r="G95" s="7"/>
@@ -27615,9 +27651,18 @@
       <c r="X95" s="7"/>
     </row>
     <row r="96" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B96" s="7"/>
-      <c r="C96" s="7"/>
-      <c r="D96" s="9"/>
+      <c r="A96" s="8">
+        <v>46282</v>
+      </c>
+      <c r="B96" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C96" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="D96" s="9">
+        <v>40000</v>
+      </c>
       <c r="E96" s="7"/>
       <c r="F96" s="7"/>
       <c r="G96" s="7"/>
@@ -39964,8 +40009,8 @@
       <c r="X589" s="7"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F93">
-    <sortCondition ref="E2:E93"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F96">
+    <sortCondition ref="E2:E96"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
@@ -40011,17 +40056,17 @@
       </c>
       <c r="B2" s="15">
         <f>'1ST TERM ACCOUNT'!AC140</f>
-        <v>48000</v>
+        <v>54000</v>
       </c>
       <c r="C2" s="15">
         <f>B2*0.7</f>
-        <v>33600</v>
+        <v>37800</v>
       </c>
       <c r="D2" s="15"/>
       <c r="E2" s="16"/>
       <c r="F2" s="15">
         <f>$C$2-D2</f>
-        <v>33600</v>
+        <v>37800</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -40037,7 +40082,7 @@
       <c r="E3" s="16"/>
       <c r="F3" s="15">
         <f>$C$2-(D2+D3)</f>
-        <v>33600</v>
+        <v>37800</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -40046,14 +40091,14 @@
       </c>
       <c r="B4" s="15">
         <f>B3-B2</f>
-        <v>144000</v>
+        <v>138000</v>
       </c>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="16"/>
       <c r="F4" s="15">
         <f>$C$2-(D2+D3+D4)</f>
-        <v>33600</v>
+        <v>37800</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -40063,7 +40108,7 @@
       <c r="E5" s="16"/>
       <c r="F5" s="15">
         <f>$C$2-(D2+D3+D4+D5)</f>
-        <v>33600</v>
+        <v>37800</v>
       </c>
       <c r="H5" s="17"/>
     </row>

</xml_diff>